<commit_message>
Added latest code for pure structural stress minimization and constraint alongside element wise poisson's ratio support and material specfic volume fractions. Also added latest code for thermo-structural compliance minimization and for thermo-structural temperature dependent compliance minimization.
</commit_message>
<xml_diff>
--- a/2-ThermoStructural/MaterialDataThermoStructural/3Materials.xlsx
+++ b/2-ThermoStructural/MaterialDataThermoStructural/3Materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\MaterialDataFiles\ThermoStructural\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METALS-main\2-ThermoStructural\MaterialDataThermoStructural\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C1F8A7-D5F2-4491-BC7D-501A4836A24F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3E8E8B-E744-4D15-8C7C-061114BAB3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1788" yWindow="2040" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="2940" windowWidth="24855" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Attributes</t>
   </si>
@@ -61,14 +61,28 @@
   </si>
   <si>
     <t>Conductivity</t>
+  </si>
+  <si>
+    <t>1/C</t>
+  </si>
+  <si>
+    <t>W/mC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -96,9 +110,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,107 +402,113 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.5546875" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="E2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>7850</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>210000000000</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>250000000</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>1.1199999999999999E-5</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>22.6</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>7800</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>200000000000</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>180000000</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>1.84E-5</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="2">
         <v>21.5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>2700</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>70000000000</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>100000000</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>2.4000000000000001E-5</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="2">
         <v>236</v>
       </c>
     </row>

</xml_diff>